<commit_message>
Update auto data track on dashboard
</commit_message>
<xml_diff>
--- a/data_dosen_dummy.xlsx
+++ b/data_dosen_dummy.xlsx
@@ -457,11 +457,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>9932601271</v>
+        <v>3410144852</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>KH. Prasetya Sitorus, S.T, M.T</t>
+          <t>Dr. Ajimin Prasasta, S.Kom, M.Kom</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -471,22 +471,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Lektor Kepala</t>
+          <t>Profesor</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>prasetya1@kampus.ac.id</t>
+          <t>ajimin1@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>5376777225</v>
+        <v>876004429</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>R. Hartaka Marpaung, S.E, M.M</t>
+          <t>Drs. Kairav Manullang, S.Kom, M.Kom</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -496,22 +496,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Lektor</t>
+          <t>Profesor</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>hartaka2@kampus.ac.id</t>
+          <t>kairav2@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3826467503</v>
+        <v>185776027</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hj. Michelle Zulaika, S.T, M.T</t>
+          <t>Ir. Salsabila Wijayanti, S.Kom, M.Kom</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -521,22 +521,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Lektor</t>
+          <t>Asisten Ahli</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>michelle3@kampus.ac.id</t>
+          <t>salsabila3@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>6939151069</v>
+        <v>2002316487</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dr. Tiara Hasanah, S.Ds, M.Ds</t>
+          <t>dr. Laras Lailasari, S.E, M.M</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -546,77 +546,77 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Profesor</t>
+          <t>Lektor Kepala</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>tiara4@kampus.ac.id</t>
+          <t>laras4@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2351330719</v>
+        <v>5125550594</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>T. Bajragin Pradana, S.Kom, M.Kom</t>
+          <t>Dr. Dina Anggraini, S.E, M.M</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Lektor Kepala</t>
+          <t>Asisten Ahli</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>bajragin5@kampus.ac.id</t>
+          <t>dina5@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>8450542978</v>
+        <v>4798430951</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>dr. Dina Suryatmi, S.E, M.M</t>
+          <t>Dt. Elon Prakasa, S.Ds, M.Ds</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Lektor</t>
+          <t>Lektor Kepala</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>dina6@kampus.ac.id</t>
+          <t>elon6@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>4236710245</v>
+        <v>1336235732</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ir. Maman Latupono, S.T, M.T</t>
+          <t>R.A. Salimah Palastri, S.Kom, M.Kom</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -626,42 +626,42 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>maman7@kampus.ac.id</t>
+          <t>salimah7@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>4282127090</v>
+        <v>5933592792</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ir. Bambang Mahendra, S.Kom, M.Kom</t>
+          <t>dr. Cindy Rahayu, S.Kom, M.Kom</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Lektor Kepala</t>
+          <t>Lektor</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>bambang8@kampus.ac.id</t>
+          <t>cindy8@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>4886616253</v>
+        <v>6871430712</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>KH. Salman Jailani, S.Kom, M.Kom</t>
+          <t>R. Jaya Simanjuntak, S.T, M.T</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -676,17 +676,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>salman9@kampus.ac.id</t>
+          <t>jaya9@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>9179606582</v>
+        <v>3628236538</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Ir. Samsul Hidayanto, S.T, M.T</t>
+          <t>R. Gantar Tampubolon, S.Kom, M.Kom</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -696,47 +696,47 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Profesor</t>
+          <t>Lektor Kepala</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>samsul10@kampus.ac.id</t>
+          <t>gantar10@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>3598051387</v>
+        <v>480531930</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Hj. Cindy Maryati, S.Kom, M.Kom</t>
+          <t>Dr. Jamal Wibowo, S.T, M.T</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Asisten Ahli</t>
+          <t>Lektor</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>cindy11@kampus.ac.id</t>
+          <t>jamal11@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>7010386305</v>
+        <v>687454040</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>drg. Paulin Riyanti, S.Ds, M.Ds</t>
+          <t>drg. Novi Padmasari, S.T, M.T</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -746,97 +746,97 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Asisten Ahli</t>
+          <t>Lektor</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>paulin12@kampus.ac.id</t>
+          <t>novi12@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1605013429</v>
+        <v>9240315641</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Dt. Prayitna Firmansyah, S.E, M.M</t>
+          <t>drg. Nilam Lailasari, S.Kom, M.Kom</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Asisten Ahli</t>
+          <t>Lektor Kepala</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>prayitna13@kampus.ac.id</t>
+          <t>nilam13@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>9657767607</v>
+        <v>6359180991</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Sutan Lurhur Tarihoran, S.E, M.M</t>
+          <t>Drs. Yulia Widiastuti, S.T, M.T</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Profesor</t>
+          <t>Lektor Kepala</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>lurhur14@kampus.ac.id</t>
+          <t>yulia14@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>6875556910</v>
+        <v>388552437</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Ir. Victoria Haryanti, S.Ds, M.Ds</t>
+          <t>Sutan Adhiarja Utama, S.Ds, M.Ds</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Lektor</t>
+          <t>Lektor Kepala</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>victoria15@kampus.ac.id</t>
+          <t>adhiarja15@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>9647601498</v>
+        <v>9567691248</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>R. Tugiman Marbun, S.Ds, M.Ds</t>
+          <t>H. Ikin Maheswara, S.E, M.M</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -846,22 +846,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Asisten Ahli</t>
+          <t>Profesor</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>tugiman16@kampus.ac.id</t>
+          <t>ikin16@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2764531336</v>
+        <v>9592933710</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>dr. Panca Gunarto, S.Ds, M.Ds</t>
+          <t>dr. Muni Hutasoit, S.Ds, M.Ds</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -871,22 +871,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Lektor Kepala</t>
+          <t>Asisten Ahli</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>panca17@kampus.ac.id</t>
+          <t>muni17@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1486484127</v>
+        <v>3785740857</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>H. Legawa Samosir, S.E, M.M</t>
+          <t>Dt. Cahyanto Permadi, S.E, M.M</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -896,22 +896,22 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Asisten Ahli</t>
+          <t>Profesor</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>legawa18@kampus.ac.id</t>
+          <t>cahyanto18@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2414853980</v>
+        <v>7053215484</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>R. Anita Astuti, S.Kom, M.Kom</t>
+          <t>Dr. Michelle Halimah, S.Ds, M.Ds</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -921,22 +921,22 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Profesor</t>
+          <t>Lektor</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>anita19@kampus.ac.id</t>
+          <t>michelle19@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>9954428191</v>
+        <v>3709860042</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>drg. Mustofa Wahyudin, S.E, M.M</t>
+          <t>Ir. Prabowo Natsir, S.Ds, M.Ds</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -946,22 +946,22 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Lektor</t>
+          <t>Lektor Kepala</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>mustofa20@kampus.ac.id</t>
+          <t>prabowo20@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>5733549454</v>
+        <v>8869725721</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>T. Naradi Prayoga, S.Kom, M.Kom</t>
+          <t>KH. Adinata Tamba, S.Kom, M.Kom</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -976,42 +976,42 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>naradi21@kampus.ac.id</t>
+          <t>adinata21@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>8672372391</v>
+        <v>5810828087</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>T. Dalimin Uwais, S.T, M.T</t>
+          <t>Puti Maida Nuraini, S.E, M.M</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Lektor</t>
+          <t>Lektor Kepala</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>dalimin22@kampus.ac.id</t>
+          <t>maida22@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>6605853023</v>
+        <v>8841982329</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>T. Galih Nugroho, S.E, M.M</t>
+          <t>R. Kurnia Natsir, S.Ds, M.Ds</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1021,22 +1021,22 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Asisten Ahli</t>
+          <t>Lektor Kepala</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>galih23@kampus.ac.id</t>
+          <t>kurnia23@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>3658686624</v>
+        <v>8194893446</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>R. Asmianto Maheswara, S.Kom, M.Kom</t>
+          <t>dr. Sakti Najmudin, S.Kom, M.Kom</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1051,32 +1051,32 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>asmianto24@kampus.ac.id</t>
+          <t>sakti24@kampus.ac.id</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>5629465644</v>
+        <v>2898116612</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>R. Salimah Purnawati, S.Ds, M.Ds</t>
+          <t>H. Mustofa Saragih, S.E, M.M</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Profesor</t>
+          <t>Asisten Ahli</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>salimah25@kampus.ac.id</t>
+          <t>mustofa25@kampus.ac.id</t>
         </is>
       </c>
     </row>

</xml_diff>